<commit_message>
fix: corrigir telefone null do João Silva na tabela backoffice - Telefone 5511911340912 estava ausente no banco de dados - Atualizado banco SQLite e confirmada planilha com dados corretos - Corrige notificações WhatsApp e e-mail do usuário joao
</commit_message>
<xml_diff>
--- a/data/backoffice/backoffice.xlsx
+++ b/data/backoffice/backoffice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maquinascomprint-my.sharepoint.com/personal/ricardo_almeida_comprint_com_br/Documents/PROJETOS/OUTROS/Programação/chatbot-whatsapp-estoque/data/backoffice/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{2CC18B3B-0087-44ED-BA23-2179E1418EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B17F45D5-C67D-47EF-BCD5-3829E17A3655}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{2CC18B3B-0087-44ED-BA23-2179E1418EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64AC0775-5421-46EB-94FE-144D52E2C490}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{003DF816-8C03-4A45-B145-3109FB5EBCDE}"/>
+    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{003DF816-8C03-4A45-B145-3109FB5EBCDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -541,6 +541,9 @@
       <c r="A4" t="s">
         <v>9</v>
       </c>
+      <c r="B4" s="1">
+        <v>5511911340912</v>
+      </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
       </c>

</xml_diff>